<commit_message>
falta arrumar cores na tabela
</commit_message>
<xml_diff>
--- a/planilhas/estoque_lab_completa.xlsx
+++ b/planilhas/estoque_lab_completa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andressluis\Desktop\Algoritmos_IPT\estoque_lab\planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CDE1A41-7419-4333-9382-5A27AF318B2C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4638FBF4-E3BC-44CC-9867-0F39E257E70D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1469" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1475" uniqueCount="561">
   <si>
     <t>Tipo</t>
   </si>
@@ -1702,6 +1702,12 @@
   </si>
   <si>
     <t>Slot da antena</t>
+  </si>
+  <si>
+    <t>COnector</t>
+  </si>
+  <si>
+    <t>BNC macho para KRE 2 vias</t>
   </si>
 </sst>
 </file>
@@ -2507,7 +2513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G258"/>
+  <dimension ref="A1:G259"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.28515625" customWidth="1"/>
@@ -4706,48 +4712,48 @@
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="20" t="s">
+        <v>559</v>
+      </c>
+      <c r="B96" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="C96" s="20" t="s">
+        <v>560</v>
+      </c>
+      <c r="D96" s="22">
+        <v>2</v>
+      </c>
+      <c r="E96" s="59" t="s">
+        <v>210</v>
+      </c>
+      <c r="F96" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G96" s="3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" s="20" t="s">
         <v>229</v>
       </c>
-      <c r="B96" s="21" t="s">
+      <c r="B97" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="C96" s="20" t="s">
+      <c r="C97" s="20" t="s">
         <v>226</v>
       </c>
-      <c r="D96" s="22">
+      <c r="D97" s="22">
         <v>1</v>
       </c>
-      <c r="E96" s="60" t="s">
+      <c r="E97" s="60" t="s">
         <v>210</v>
       </c>
-      <c r="F96" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G96" s="18" t="s">
+      <c r="F97" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G97" s="18" t="s">
         <v>231</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A97" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="B97" s="23" t="s">
-        <v>241</v>
-      </c>
-      <c r="C97" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="D97" s="10">
-        <v>10</v>
-      </c>
-      <c r="E97" s="61" t="s">
-        <v>232</v>
-      </c>
-      <c r="F97" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G97" s="3" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
@@ -4758,7 +4764,7 @@
         <v>241</v>
       </c>
       <c r="C98" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D98" s="10">
         <v>10</v>
@@ -4775,16 +4781,16 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B99" s="23" t="s">
         <v>241</v>
       </c>
       <c r="C99" s="10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D99" s="10">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E99" s="61" t="s">
         <v>232</v>
@@ -4797,48 +4803,50 @@
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A100" s="20" t="s">
+      <c r="A100" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="B100" s="23" t="s">
+        <v>241</v>
+      </c>
+      <c r="C100" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="D100" s="10">
+        <v>5</v>
+      </c>
+      <c r="E100" s="61" t="s">
+        <v>232</v>
+      </c>
+      <c r="F100" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G100" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A101" s="20" t="s">
         <v>240</v>
       </c>
-      <c r="B100" s="24" t="s">
+      <c r="B101" s="24" t="s">
         <v>241</v>
       </c>
-      <c r="C100" s="22" t="s">
+      <c r="C101" s="22" t="s">
         <v>237</v>
       </c>
-      <c r="D100" s="22">
+      <c r="D101" s="22">
         <v>7</v>
       </c>
-      <c r="E100" s="62" t="s">
+      <c r="E101" s="62" t="s">
         <v>232</v>
       </c>
-      <c r="F100" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G100" s="18" t="s">
+      <c r="F101" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G101" s="18" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A101" s="16" t="s">
-        <v>242</v>
-      </c>
-      <c r="B101" s="25" t="s">
-        <v>248</v>
-      </c>
-      <c r="C101" s="10" t="s">
-        <v>243</v>
-      </c>
-      <c r="D101" s="10">
-        <v>2</v>
-      </c>
-      <c r="E101" s="63" t="s">
-        <v>247</v>
-      </c>
-      <c r="F101" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G101" s="1"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="16" t="s">
@@ -4848,10 +4856,10 @@
         <v>248</v>
       </c>
       <c r="C102" s="10" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D102" s="10">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E102" s="63" t="s">
         <v>247</v>
@@ -4869,10 +4877,10 @@
         <v>248</v>
       </c>
       <c r="C103" s="10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D103" s="10">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E103" s="63" t="s">
         <v>247</v>
@@ -4883,46 +4891,46 @@
       <c r="G103" s="1"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A104" s="20" t="s">
+      <c r="A104" s="16" t="s">
         <v>242</v>
       </c>
-      <c r="B104" s="26" t="s">
+      <c r="B104" s="25" t="s">
         <v>248</v>
       </c>
-      <c r="C104" s="22" t="s">
+      <c r="C104" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="D104" s="10">
+        <v>11</v>
+      </c>
+      <c r="E104" s="63" t="s">
+        <v>247</v>
+      </c>
+      <c r="F104" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G104" s="1"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="B105" s="26" t="s">
+        <v>248</v>
+      </c>
+      <c r="C105" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="D104" s="22">
+      <c r="D105" s="22">
         <v>4</v>
       </c>
-      <c r="E104" s="64" t="s">
+      <c r="E105" s="64" t="s">
         <v>247</v>
       </c>
-      <c r="F104" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G104" s="27"/>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A105" s="16" t="s">
-        <v>258</v>
-      </c>
-      <c r="B105" s="28" t="s">
-        <v>258</v>
-      </c>
-      <c r="C105" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="D105" s="10">
-        <v>34</v>
-      </c>
-      <c r="E105" s="65" t="s">
-        <v>249</v>
-      </c>
-      <c r="F105" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G105" s="1"/>
+      <c r="F105" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G105" s="27"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="16" t="s">
@@ -4932,10 +4940,10 @@
         <v>258</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D106" s="10">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E106" s="65" t="s">
         <v>249</v>
@@ -4953,10 +4961,10 @@
         <v>258</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D107" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E107" s="65" t="s">
         <v>249</v>
@@ -4974,7 +4982,7 @@
         <v>258</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D108" s="10">
         <v>1</v>
@@ -4995,7 +5003,7 @@
         <v>258</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D109" s="10">
         <v>1</v>
@@ -5016,7 +5024,7 @@
         <v>258</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D110" s="10">
         <v>1</v>
@@ -5037,10 +5045,10 @@
         <v>258</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D111" s="10">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E111" s="65" t="s">
         <v>249</v>
@@ -5051,46 +5059,46 @@
       <c r="G111" s="1"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A112" s="20" t="s">
+      <c r="A112" s="16" t="s">
         <v>258</v>
       </c>
-      <c r="B112" s="29" t="s">
+      <c r="B112" s="28" t="s">
         <v>258</v>
       </c>
-      <c r="C112" s="18" t="s">
+      <c r="C112" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D112" s="10">
+        <v>22</v>
+      </c>
+      <c r="E112" s="65" t="s">
+        <v>249</v>
+      </c>
+      <c r="F112" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G112" s="1"/>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A113" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="B113" s="29" t="s">
+        <v>258</v>
+      </c>
+      <c r="C113" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="D112" s="22">
+      <c r="D113" s="22">
         <v>3</v>
       </c>
-      <c r="E112" s="66" t="s">
+      <c r="E113" s="66" t="s">
         <v>249</v>
       </c>
-      <c r="F112" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G112" s="27"/>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A113" s="16" t="s">
-        <v>259</v>
-      </c>
-      <c r="B113" s="16" t="s">
-        <v>259</v>
-      </c>
-      <c r="C113" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="D113" s="10">
-        <v>3</v>
-      </c>
-      <c r="E113" s="67" t="s">
-        <v>260</v>
-      </c>
-      <c r="F113" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G113" s="1"/>
+      <c r="F113" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G113" s="27"/>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="16" t="s">
@@ -5100,10 +5108,10 @@
         <v>259</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D114" s="10">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E114" s="67" t="s">
         <v>260</v>
@@ -5121,10 +5129,10 @@
         <v>259</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D115" s="10">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E115" s="67" t="s">
         <v>260</v>
@@ -5142,10 +5150,10 @@
         <v>259</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D116" s="10">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E116" s="67" t="s">
         <v>260</v>
@@ -5163,10 +5171,10 @@
         <v>259</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D117" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E117" s="67" t="s">
         <v>260</v>
@@ -5184,10 +5192,10 @@
         <v>259</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="D118" s="11">
-        <v>2</v>
+        <v>265</v>
+      </c>
+      <c r="D118" s="10">
+        <v>3</v>
       </c>
       <c r="E118" s="67" t="s">
         <v>260</v>
@@ -5199,19 +5207,19 @@
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="16" t="s">
-        <v>274</v>
-      </c>
-      <c r="B119" s="23" t="s">
-        <v>267</v>
+        <v>259</v>
+      </c>
+      <c r="B119" s="16" t="s">
+        <v>259</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="D119" s="10">
-        <v>4</v>
-      </c>
-      <c r="E119" s="36" t="s">
-        <v>273</v>
+        <v>266</v>
+      </c>
+      <c r="D119" s="11">
+        <v>2</v>
+      </c>
+      <c r="E119" s="67" t="s">
+        <v>260</v>
       </c>
       <c r="F119" s="5" t="s">
         <v>15</v>
@@ -5220,16 +5228,16 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="16" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B120" s="23" t="s">
         <v>267</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D120" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E120" s="36" t="s">
         <v>273</v>
@@ -5241,16 +5249,16 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="16" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B121" s="23" t="s">
         <v>267</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D121" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E121" s="36" t="s">
         <v>273</v>
@@ -5262,16 +5270,16 @@
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="16" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B122" s="23" t="s">
         <v>267</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D122" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E122" s="36" t="s">
         <v>273</v>
@@ -5282,46 +5290,46 @@
       <c r="G122" s="1"/>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A123" s="20" t="s">
+      <c r="A123" s="16" t="s">
+        <v>277</v>
+      </c>
+      <c r="B123" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D123" s="10">
+        <v>2</v>
+      </c>
+      <c r="E123" s="36" t="s">
+        <v>273</v>
+      </c>
+      <c r="F123" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G123" s="1"/>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A124" s="20" t="s">
         <v>278</v>
       </c>
-      <c r="B123" s="24" t="s">
+      <c r="B124" s="24" t="s">
         <v>267</v>
       </c>
-      <c r="C123" s="30" t="s">
+      <c r="C124" s="30" t="s">
         <v>272</v>
       </c>
-      <c r="D123" s="17">
+      <c r="D124" s="17">
         <v>24</v>
       </c>
-      <c r="E123" s="55" t="s">
+      <c r="E124" s="55" t="s">
         <v>273</v>
       </c>
-      <c r="F123" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G123" s="27"/>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A124" s="16" t="s">
-        <v>280</v>
-      </c>
-      <c r="B124" s="31" t="s">
-        <v>279</v>
-      </c>
-      <c r="C124" s="8" t="s">
-        <v>281</v>
-      </c>
-      <c r="D124" s="10">
-        <v>23</v>
-      </c>
-      <c r="E124" s="68" t="s">
-        <v>294</v>
-      </c>
-      <c r="F124" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G124" s="1"/>
+      <c r="F124" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G124" s="27"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="16" t="s">
@@ -5331,10 +5339,10 @@
         <v>279</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D125" s="10">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E125" s="68" t="s">
         <v>294</v>
@@ -5352,7 +5360,7 @@
         <v>279</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D126" s="10">
         <v>4</v>
@@ -5373,10 +5381,10 @@
         <v>279</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D127" s="10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E127" s="68" t="s">
         <v>294</v>
@@ -5394,10 +5402,10 @@
         <v>279</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D128" s="10">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E128" s="68" t="s">
         <v>294</v>
@@ -5415,10 +5423,10 @@
         <v>279</v>
       </c>
       <c r="C129" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D129" s="10">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E129" s="68" t="s">
         <v>294</v>
@@ -5436,10 +5444,10 @@
         <v>279</v>
       </c>
       <c r="C130" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D130" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E130" s="68" t="s">
         <v>294</v>
@@ -5457,10 +5465,10 @@
         <v>279</v>
       </c>
       <c r="C131" s="8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D131" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E131" s="68" t="s">
         <v>294</v>
@@ -5478,10 +5486,10 @@
         <v>279</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D132" s="10">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E132" s="68" t="s">
         <v>294</v>
@@ -5499,10 +5507,10 @@
         <v>279</v>
       </c>
       <c r="C133" s="8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D133" s="10">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E133" s="68" t="s">
         <v>294</v>
@@ -5520,7 +5528,7 @@
         <v>279</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D134" s="10">
         <v>2</v>
@@ -5541,10 +5549,10 @@
         <v>279</v>
       </c>
       <c r="C135" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D135" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E135" s="68" t="s">
         <v>294</v>
@@ -5555,56 +5563,56 @@
       <c r="G135" s="1"/>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A136" s="20" t="s">
+      <c r="A136" s="16" t="s">
         <v>280</v>
       </c>
-      <c r="B136" s="32" t="s">
+      <c r="B136" s="31" t="s">
         <v>279</v>
       </c>
-      <c r="C136" s="14" t="s">
+      <c r="C136" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="D136" s="10">
+        <v>1</v>
+      </c>
+      <c r="E136" s="68" t="s">
+        <v>294</v>
+      </c>
+      <c r="F136" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G136" s="1"/>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A137" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="B137" s="32" t="s">
+        <v>279</v>
+      </c>
+      <c r="C137" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="D136" s="17">
+      <c r="D137" s="17">
         <v>1</v>
       </c>
-      <c r="E136" s="69" t="s">
+      <c r="E137" s="69" t="s">
         <v>294</v>
       </c>
-      <c r="F136" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G136" s="27"/>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A137" s="16" t="s">
-        <v>304</v>
-      </c>
-      <c r="B137" s="33" t="s">
-        <v>295</v>
-      </c>
-      <c r="C137" s="8" t="s">
-        <v>296</v>
-      </c>
-      <c r="D137" s="10">
-        <v>20</v>
-      </c>
-      <c r="E137" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="F137" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G137" s="1"/>
+      <c r="F137" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G137" s="27"/>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" s="16" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B138" s="33" t="s">
         <v>295</v>
       </c>
       <c r="C138" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D138" s="10">
         <v>20</v>
@@ -5619,16 +5627,16 @@
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" s="16" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B139" s="33" t="s">
         <v>295</v>
       </c>
       <c r="C139" s="8" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D139" s="10">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E139" s="3" t="s">
         <v>312</v>
@@ -5640,16 +5648,16 @@
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" s="16" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B140" s="33" t="s">
         <v>295</v>
       </c>
       <c r="C140" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D140" s="10">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E140" s="3" t="s">
         <v>312</v>
@@ -5661,16 +5669,16 @@
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" s="16" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B141" s="33" t="s">
         <v>295</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D141" s="10">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E141" s="3" t="s">
         <v>312</v>
@@ -5682,16 +5690,16 @@
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A142" s="16" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B142" s="33" t="s">
         <v>295</v>
       </c>
       <c r="C142" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D142" s="10">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E142" s="3" t="s">
         <v>312</v>
@@ -5703,13 +5711,13 @@
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A143" s="16" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B143" s="33" t="s">
         <v>295</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D143" s="10">
         <v>20</v>
@@ -5723,59 +5731,59 @@
       <c r="G143" s="1"/>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A144" s="20" t="s">
+      <c r="A144" s="16" t="s">
+        <v>310</v>
+      </c>
+      <c r="B144" s="33" t="s">
+        <v>295</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>302</v>
+      </c>
+      <c r="D144" s="10">
+        <v>20</v>
+      </c>
+      <c r="E144" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="F144" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G144" s="1"/>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A145" s="20" t="s">
         <v>311</v>
       </c>
-      <c r="B144" s="34" t="s">
+      <c r="B145" s="34" t="s">
         <v>295</v>
       </c>
-      <c r="C144" s="14" t="s">
+      <c r="C145" s="14" t="s">
         <v>303</v>
       </c>
-      <c r="D144" s="17">
+      <c r="D145" s="17">
         <v>20</v>
       </c>
-      <c r="E144" s="18" t="s">
+      <c r="E145" s="18" t="s">
         <v>312</v>
       </c>
-      <c r="F144" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G144" s="27"/>
-    </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A145" s="16" t="s">
+      <c r="F145" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G145" s="27"/>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A146" s="16" t="s">
         <v>342</v>
-      </c>
-      <c r="B145" s="35" t="s">
-        <v>313</v>
-      </c>
-      <c r="C145" s="38" t="s">
-        <v>314</v>
-      </c>
-      <c r="D145" s="38">
-        <v>12</v>
-      </c>
-      <c r="E145" s="36" t="s">
-        <v>344</v>
-      </c>
-      <c r="F145" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G145" s="2"/>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A146" s="10" t="s">
-        <v>315</v>
       </c>
       <c r="B146" s="35" t="s">
         <v>313</v>
       </c>
-      <c r="C146" s="10" t="s">
-        <v>315</v>
+      <c r="C146" s="38" t="s">
+        <v>314</v>
       </c>
       <c r="D146" s="38">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E146" s="36" t="s">
         <v>344</v>
@@ -5783,22 +5791,20 @@
       <c r="F146" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G146" s="2" t="s">
-        <v>345</v>
-      </c>
+      <c r="G146" s="2"/>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A147" s="16" t="s">
-        <v>491</v>
+      <c r="A147" s="10" t="s">
+        <v>315</v>
       </c>
       <c r="B147" s="35" t="s">
-        <v>346</v>
-      </c>
-      <c r="C147" s="38" t="s">
-        <v>316</v>
+        <v>313</v>
+      </c>
+      <c r="C147" s="10" t="s">
+        <v>315</v>
       </c>
       <c r="D147" s="38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E147" s="36" t="s">
         <v>344</v>
@@ -5812,13 +5818,13 @@
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="16" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B148" s="35" t="s">
         <v>346</v>
       </c>
-      <c r="C148" s="10" t="s">
-        <v>317</v>
+      <c r="C148" s="38" t="s">
+        <v>316</v>
       </c>
       <c r="D148" s="38">
         <v>1</v>
@@ -5835,13 +5841,13 @@
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="16" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B149" s="35" t="s">
         <v>346</v>
       </c>
       <c r="C149" s="10" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D149" s="38">
         <v>1</v>
@@ -5858,16 +5864,16 @@
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="16" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B150" s="35" t="s">
         <v>346</v>
       </c>
       <c r="C150" s="10" t="s">
-        <v>319</v>
-      </c>
-      <c r="D150" s="10">
-        <v>2</v>
+        <v>318</v>
+      </c>
+      <c r="D150" s="38">
+        <v>1</v>
       </c>
       <c r="E150" s="36" t="s">
         <v>344</v>
@@ -5881,16 +5887,16 @@
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="16" t="s">
-        <v>347</v>
+        <v>488</v>
       </c>
       <c r="B151" s="35" t="s">
-        <v>313</v>
+        <v>346</v>
       </c>
       <c r="C151" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D151" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E151" s="36" t="s">
         <v>344</v>
@@ -5899,18 +5905,18 @@
         <v>15</v>
       </c>
       <c r="G151" s="2" t="s">
-        <v>367</v>
+        <v>345</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="16" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B152" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C152" s="10" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D152" s="10">
         <v>1</v>
@@ -5927,13 +5933,13 @@
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="16" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B153" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C153" s="10" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D153" s="10">
         <v>1</v>
@@ -5950,34 +5956,36 @@
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="16" t="s">
-        <v>499</v>
+        <v>349</v>
       </c>
       <c r="B154" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C154" s="10" t="s">
-        <v>500</v>
+        <v>322</v>
       </c>
       <c r="D154" s="10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E154" s="36" t="s">
         <v>344</v>
       </c>
-      <c r="F154" s="5"/>
+      <c r="F154" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="G154" s="2" t="s">
-        <v>501</v>
+        <v>367</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="16" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="B155" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C155" s="10" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="D155" s="10">
         <v>4</v>
@@ -5985,25 +5993,23 @@
       <c r="E155" s="36" t="s">
         <v>344</v>
       </c>
-      <c r="F155" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G155" s="10" t="s">
-        <v>498</v>
+      <c r="F155" s="5"/>
+      <c r="G155" s="2" t="s">
+        <v>501</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A156" s="2" t="s">
-        <v>354</v>
+      <c r="A156" s="16" t="s">
+        <v>496</v>
       </c>
       <c r="B156" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C156" s="10" t="s">
-        <v>323</v>
+        <v>497</v>
       </c>
       <c r="D156" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E156" s="36" t="s">
         <v>344</v>
@@ -6011,19 +6017,19 @@
       <c r="F156" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G156" s="2" t="s">
-        <v>367</v>
+      <c r="G156" s="10" t="s">
+        <v>498</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B157" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C157" s="10" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D157" s="10">
         <v>1</v>
@@ -6040,13 +6046,13 @@
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="B158" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C158" s="10" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D158" s="10">
         <v>1</v>
@@ -6063,13 +6069,13 @@
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B159" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C159" s="10" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D159" s="10">
         <v>1</v>
@@ -6086,13 +6092,13 @@
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B160" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C160" s="10" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D160" s="10">
         <v>1</v>
@@ -6109,13 +6115,13 @@
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B161" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C161" s="10" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D161" s="10">
         <v>1</v>
@@ -6132,13 +6138,13 @@
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B162" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C162" s="10" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D162" s="10">
         <v>1</v>
@@ -6155,13 +6161,13 @@
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B163" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C163" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D163" s="10">
         <v>1</v>
@@ -6178,13 +6184,13 @@
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B164" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C164" s="10" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D164" s="10">
         <v>1</v>
@@ -6201,16 +6207,16 @@
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
-        <v>332</v>
+        <v>362</v>
       </c>
       <c r="B165" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C165" s="10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D165" s="10">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E165" s="36" t="s">
         <v>344</v>
@@ -6219,65 +6225,67 @@
         <v>15</v>
       </c>
       <c r="G165" s="2" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="166" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A166" s="10" t="s">
-        <v>363</v>
+        <v>367</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A166" s="2" t="s">
+        <v>332</v>
       </c>
       <c r="B166" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C166" s="10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D166" s="10">
-        <v>1</v>
-      </c>
-      <c r="E166" s="37" t="s">
+        <v>5</v>
+      </c>
+      <c r="E166" s="36" t="s">
         <v>344</v>
       </c>
       <c r="F166" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G166" s="71" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A167" s="2" t="s">
-        <v>364</v>
+      <c r="G166" s="2" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A167" s="10" t="s">
+        <v>363</v>
       </c>
       <c r="B167" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C167" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D167" s="10">
-        <v>2</v>
-      </c>
-      <c r="E167" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="E167" s="37" t="s">
         <v>344</v>
       </c>
       <c r="F167" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G167" s="72"/>
-    </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G167" s="71" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B168" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C168" s="10" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D168" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E168" s="36" t="s">
         <v>344</v>
@@ -6289,16 +6297,16 @@
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B169" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C169" s="10" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D169" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E169" s="36" t="s">
         <v>344</v>
@@ -6306,17 +6314,17 @@
       <c r="F169" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G169" s="73"/>
+      <c r="G169" s="72"/>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A170" s="16" t="s">
-        <v>351</v>
+      <c r="A170" s="2" t="s">
+        <v>366</v>
       </c>
       <c r="B170" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C170" s="10" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D170" s="10">
         <v>1</v>
@@ -6327,22 +6335,20 @@
       <c r="F170" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G170" s="2" t="s">
-        <v>367</v>
-      </c>
+      <c r="G170" s="73"/>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="16" t="s">
-        <v>493</v>
+        <v>351</v>
       </c>
       <c r="B171" s="35" t="s">
-        <v>346</v>
+        <v>313</v>
       </c>
       <c r="C171" s="10" t="s">
-        <v>493</v>
+        <v>337</v>
       </c>
       <c r="D171" s="10">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E171" s="36" t="s">
         <v>344</v>
@@ -6351,21 +6357,21 @@
         <v>15</v>
       </c>
       <c r="G171" s="2" t="s">
-        <v>494</v>
+        <v>367</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="16" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="B172" s="35" t="s">
         <v>346</v>
       </c>
       <c r="C172" s="10" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="D172" s="10">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="E172" s="36" t="s">
         <v>344</v>
@@ -6374,21 +6380,21 @@
         <v>15</v>
       </c>
       <c r="G172" s="2" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="16" t="s">
-        <v>352</v>
+        <v>486</v>
       </c>
       <c r="B173" s="35" t="s">
-        <v>313</v>
+        <v>346</v>
       </c>
       <c r="C173" s="10" t="s">
-        <v>338</v>
+        <v>487</v>
       </c>
       <c r="D173" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E173" s="36" t="s">
         <v>344</v>
@@ -6396,20 +6402,22 @@
       <c r="F173" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G173" s="2"/>
+      <c r="G173" s="2" t="s">
+        <v>492</v>
+      </c>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="16" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B174" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C174" s="10" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D174" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E174" s="36" t="s">
         <v>344</v>
@@ -6421,13 +6429,13 @@
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="16" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="B175" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C175" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D175" s="10">
         <v>1</v>
@@ -6442,13 +6450,13 @@
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="16" t="s">
-        <v>495</v>
+        <v>355</v>
       </c>
       <c r="B176" s="35" t="s">
-        <v>346</v>
+        <v>313</v>
       </c>
       <c r="C176" s="10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D176" s="10">
         <v>1</v>
@@ -6459,45 +6467,43 @@
       <c r="F176" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G176" s="2" t="s">
-        <v>345</v>
-      </c>
+      <c r="G176" s="2"/>
     </row>
     <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" s="16" t="s">
-        <v>379</v>
+        <v>495</v>
       </c>
       <c r="B177" s="35" t="s">
-        <v>313</v>
+        <v>346</v>
       </c>
       <c r="C177" s="10" t="s">
-        <v>370</v>
+        <v>341</v>
       </c>
       <c r="D177" s="10">
-        <v>5</v>
-      </c>
-      <c r="E177" s="39" t="s">
-        <v>388</v>
+        <v>1</v>
+      </c>
+      <c r="E177" s="36" t="s">
+        <v>344</v>
       </c>
       <c r="F177" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G177" s="2" t="s">
-        <v>502</v>
+        <v>345</v>
       </c>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" s="16" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B178" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C178" s="10" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D178" s="10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E178" s="39" t="s">
         <v>388</v>
@@ -6506,21 +6512,21 @@
         <v>15</v>
       </c>
       <c r="G178" s="2" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" s="16" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B179" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C179" s="10" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D179" s="10">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E179" s="39" t="s">
         <v>388</v>
@@ -6529,21 +6535,21 @@
         <v>15</v>
       </c>
       <c r="G179" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" s="16" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B180" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C180" s="10" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="D180" s="10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E180" s="39" t="s">
         <v>388</v>
@@ -6552,21 +6558,21 @@
         <v>15</v>
       </c>
       <c r="G180" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" s="16" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B181" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C181" s="10" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D181" s="10">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E181" s="39" t="s">
         <v>388</v>
@@ -6575,21 +6581,21 @@
         <v>15</v>
       </c>
       <c r="G181" s="2" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" s="16" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B182" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C182" s="10" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D182" s="10">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E182" s="39" t="s">
         <v>388</v>
@@ -6598,21 +6604,21 @@
         <v>15</v>
       </c>
       <c r="G182" s="2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" s="16" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B183" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C183" s="10" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D183" s="10">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E183" s="39" t="s">
         <v>388</v>
@@ -6621,21 +6627,21 @@
         <v>15</v>
       </c>
       <c r="G183" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" s="16" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B184" s="35" t="s">
         <v>313</v>
       </c>
       <c r="C184" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D184" s="10">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E184" s="39" t="s">
         <v>388</v>
@@ -6644,67 +6650,67 @@
         <v>15</v>
       </c>
       <c r="G184" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A185" s="20" t="s">
-        <v>387</v>
+      <c r="A185" s="16" t="s">
+        <v>386</v>
       </c>
       <c r="B185" s="35" t="s">
         <v>313</v>
       </c>
-      <c r="C185" s="17" t="s">
+      <c r="C185" s="10" t="s">
+        <v>377</v>
+      </c>
+      <c r="D185" s="10">
+        <v>8</v>
+      </c>
+      <c r="E185" s="39" t="s">
+        <v>388</v>
+      </c>
+      <c r="F185" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G185" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A186" s="20" t="s">
+        <v>387</v>
+      </c>
+      <c r="B186" s="35" t="s">
+        <v>313</v>
+      </c>
+      <c r="C186" s="17" t="s">
         <v>378</v>
       </c>
-      <c r="D185" s="17">
+      <c r="D186" s="17">
         <v>7</v>
       </c>
-      <c r="E185" s="40" t="s">
+      <c r="E186" s="40" t="s">
         <v>388</v>
       </c>
-      <c r="F185" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G185" s="2" t="s">
+      <c r="F186" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G186" s="2" t="s">
         <v>510</v>
-      </c>
-    </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A186" s="10" t="s">
-        <v>390</v>
-      </c>
-      <c r="B186" s="41" t="s">
-        <v>389</v>
-      </c>
-      <c r="C186" s="10" t="s">
-        <v>390</v>
-      </c>
-      <c r="D186" s="10">
-        <v>14</v>
-      </c>
-      <c r="E186" s="42" t="s">
-        <v>403</v>
-      </c>
-      <c r="F186" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G186" s="1" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" s="10" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B187" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C187" s="10" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D187" s="10">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E187" s="42" t="s">
         <v>403</v>
@@ -6713,18 +6719,18 @@
         <v>15</v>
       </c>
       <c r="G187" s="1" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" s="10" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B188" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C188" s="10" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D188" s="10">
         <v>4</v>
@@ -6736,21 +6742,21 @@
         <v>15</v>
       </c>
       <c r="G188" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" s="10" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B189" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C189" s="10" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D189" s="10">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E189" s="42" t="s">
         <v>403</v>
@@ -6759,21 +6765,21 @@
         <v>15</v>
       </c>
       <c r="G189" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B190" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C190" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D190" s="10">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E190" s="42" t="s">
         <v>403</v>
@@ -6782,21 +6788,21 @@
         <v>15</v>
       </c>
       <c r="G190" s="1" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B191" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C191" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D191" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E191" s="42" t="s">
         <v>403</v>
@@ -6805,21 +6811,21 @@
         <v>15</v>
       </c>
       <c r="G191" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" s="10" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B192" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C192" s="10" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D192" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E192" s="42" t="s">
         <v>403</v>
@@ -6828,21 +6834,21 @@
         <v>15</v>
       </c>
       <c r="G192" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" s="10" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B193" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C193" s="10" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D193" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E193" s="42" t="s">
         <v>403</v>
@@ -6851,21 +6857,21 @@
         <v>15</v>
       </c>
       <c r="G193" s="1" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B194" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C194" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D194" s="10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E194" s="42" t="s">
         <v>403</v>
@@ -6879,16 +6885,16 @@
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B195" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C195" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="D195" s="10">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E195" s="42" t="s">
         <v>403</v>
@@ -6897,21 +6903,21 @@
         <v>15</v>
       </c>
       <c r="G195" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B196" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C196" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D196" s="10">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E196" s="42" t="s">
         <v>403</v>
@@ -6920,21 +6926,21 @@
         <v>15</v>
       </c>
       <c r="G196" s="1" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B197" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C197" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D197" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E197" s="42" t="s">
         <v>403</v>
@@ -6943,21 +6949,21 @@
         <v>15</v>
       </c>
       <c r="G197" s="1" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" s="10" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B198" s="41" t="s">
         <v>389</v>
       </c>
       <c r="C198" s="10" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D198" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E198" s="42" t="s">
         <v>403</v>
@@ -6966,53 +6972,53 @@
         <v>15</v>
       </c>
       <c r="G198" s="1" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A199" s="10" t="s">
+        <v>402</v>
+      </c>
+      <c r="B199" s="41" t="s">
+        <v>389</v>
+      </c>
+      <c r="C199" s="10" t="s">
+        <v>402</v>
+      </c>
+      <c r="D199" s="10">
+        <v>1</v>
+      </c>
+      <c r="E199" s="42" t="s">
+        <v>403</v>
+      </c>
+      <c r="F199" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G199" s="1" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A199" s="16" t="s">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A200" s="16" t="s">
         <v>556</v>
       </c>
-      <c r="B199" s="70" t="s">
+      <c r="B200" s="70" t="s">
         <v>556</v>
       </c>
-      <c r="C199" s="10" t="s">
+      <c r="C200" s="10" t="s">
         <v>555</v>
       </c>
-      <c r="D199" s="10">
+      <c r="D200" s="10">
         <v>14</v>
       </c>
-      <c r="E199" s="42" t="s">
+      <c r="E200" s="42" t="s">
         <v>557</v>
       </c>
-      <c r="F199" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G199" s="1" t="s">
+      <c r="F200" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G200" s="1" t="s">
         <v>558</v>
-      </c>
-    </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A200" s="11" t="s">
-        <v>404</v>
-      </c>
-      <c r="B200" s="43" t="s">
-        <v>410</v>
-      </c>
-      <c r="C200" s="10" t="s">
-        <v>405</v>
-      </c>
-      <c r="D200" s="10">
-        <v>2</v>
-      </c>
-      <c r="E200" s="44" t="s">
-        <v>411</v>
-      </c>
-      <c r="F200" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G200" s="1" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.25">
@@ -7023,10 +7029,10 @@
         <v>410</v>
       </c>
       <c r="C201" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D201" s="10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E201" s="44" t="s">
         <v>411</v>
@@ -7035,7 +7041,7 @@
         <v>15</v>
       </c>
       <c r="G201" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="202" spans="1:7" x14ac:dyDescent="0.25">
@@ -7046,10 +7052,10 @@
         <v>410</v>
       </c>
       <c r="C202" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D202" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E202" s="44" t="s">
         <v>411</v>
@@ -7058,7 +7064,7 @@
         <v>15</v>
       </c>
       <c r="G202" s="1" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
     </row>
     <row r="203" spans="1:7" x14ac:dyDescent="0.25">
@@ -7068,10 +7074,10 @@
       <c r="B203" s="43" t="s">
         <v>410</v>
       </c>
-      <c r="C203" s="11" t="s">
-        <v>408</v>
-      </c>
-      <c r="D203" s="11">
+      <c r="C203" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="D203" s="10">
         <v>1</v>
       </c>
       <c r="E203" s="44" t="s">
@@ -7081,7 +7087,7 @@
         <v>15</v>
       </c>
       <c r="G203" s="1" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="204" spans="1:7" x14ac:dyDescent="0.25">
@@ -7092,7 +7098,7 @@
         <v>410</v>
       </c>
       <c r="C204" s="11" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="D204" s="11">
         <v>1</v>
@@ -7103,43 +7109,43 @@
       <c r="F204" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G204" s="1"/>
+      <c r="G204" s="1" t="s">
+        <v>532</v>
+      </c>
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" s="11" t="s">
-        <v>512</v>
-      </c>
-      <c r="B205" s="50" t="s">
-        <v>428</v>
-      </c>
-      <c r="C205" s="10" t="s">
-        <v>413</v>
-      </c>
-      <c r="D205" s="10">
-        <v>4</v>
-      </c>
-      <c r="E205" s="51" t="s">
-        <v>435</v>
+        <v>404</v>
+      </c>
+      <c r="B205" s="43" t="s">
+        <v>410</v>
+      </c>
+      <c r="C205" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="D205" s="11">
+        <v>1</v>
+      </c>
+      <c r="E205" s="44" t="s">
+        <v>411</v>
       </c>
       <c r="F205" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G205" s="1" t="s">
-        <v>547</v>
-      </c>
+      <c r="G205" s="1"/>
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" s="11" t="s">
-        <v>412</v>
-      </c>
-      <c r="B206" s="33" t="s">
-        <v>429</v>
+        <v>512</v>
+      </c>
+      <c r="B206" s="50" t="s">
+        <v>428</v>
       </c>
       <c r="C206" s="10" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D206" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E206" s="51" t="s">
         <v>435</v>
@@ -7148,21 +7154,21 @@
         <v>15</v>
       </c>
       <c r="G206" s="1" t="s">
-        <v>533</v>
+        <v>547</v>
       </c>
     </row>
     <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B207" s="49" t="s">
-        <v>430</v>
-      </c>
-      <c r="C207" s="11" t="s">
-        <v>415</v>
-      </c>
-      <c r="D207" s="11">
-        <v>2</v>
+      <c r="B207" s="33" t="s">
+        <v>429</v>
+      </c>
+      <c r="C207" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="D207" s="10">
+        <v>1</v>
       </c>
       <c r="E207" s="51" t="s">
         <v>435</v>
@@ -7171,21 +7177,21 @@
         <v>15</v>
       </c>
       <c r="G207" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B208" s="45" t="s">
-        <v>433</v>
+      <c r="B208" s="49" t="s">
+        <v>430</v>
       </c>
       <c r="C208" s="11" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D208" s="11">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E208" s="51" t="s">
         <v>435</v>
@@ -7194,21 +7200,21 @@
         <v>15</v>
       </c>
       <c r="G208" s="1" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B209" s="33" t="s">
-        <v>429</v>
-      </c>
-      <c r="C209" s="10" t="s">
-        <v>417</v>
-      </c>
-      <c r="D209" s="10">
-        <v>9</v>
+      <c r="B209" s="45" t="s">
+        <v>433</v>
+      </c>
+      <c r="C209" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="D209" s="11">
+        <v>10</v>
       </c>
       <c r="E209" s="51" t="s">
         <v>435</v>
@@ -7217,7 +7223,7 @@
         <v>15</v>
       </c>
       <c r="G209" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.25">
@@ -7228,10 +7234,10 @@
         <v>429</v>
       </c>
       <c r="C210" s="10" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D210" s="10">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E210" s="51" t="s">
         <v>435</v>
@@ -7251,10 +7257,10 @@
         <v>429</v>
       </c>
       <c r="C211" s="10" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D211" s="10">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E211" s="51" t="s">
         <v>435</v>
@@ -7263,7 +7269,7 @@
         <v>15</v>
       </c>
       <c r="G211" s="1" t="s">
-        <v>535</v>
+        <v>528</v>
       </c>
     </row>
     <row r="212" spans="1:7" x14ac:dyDescent="0.25">
@@ -7273,10 +7279,10 @@
       <c r="B212" s="33" t="s">
         <v>429</v>
       </c>
-      <c r="C212" s="11" t="s">
-        <v>420</v>
-      </c>
-      <c r="D212" s="11">
+      <c r="C212" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D212" s="10">
         <v>1</v>
       </c>
       <c r="E212" s="51" t="s">
@@ -7286,7 +7292,7 @@
         <v>15</v>
       </c>
       <c r="G212" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.25">
@@ -7297,7 +7303,7 @@
         <v>429</v>
       </c>
       <c r="C213" s="11" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D213" s="11">
         <v>1</v>
@@ -7309,21 +7315,21 @@
         <v>15</v>
       </c>
       <c r="G213" s="1" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B214" s="45" t="s">
-        <v>431</v>
-      </c>
-      <c r="C214" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="D214" s="10">
-        <v>5</v>
+      <c r="B214" s="33" t="s">
+        <v>429</v>
+      </c>
+      <c r="C214" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="D214" s="11">
+        <v>1</v>
       </c>
       <c r="E214" s="51" t="s">
         <v>435</v>
@@ -7332,7 +7338,7 @@
         <v>15</v>
       </c>
       <c r="G214" s="1" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.25">
@@ -7340,13 +7346,13 @@
         <v>412</v>
       </c>
       <c r="B215" s="45" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C215" s="10" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D215" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E215" s="51" t="s">
         <v>435</v>
@@ -7355,18 +7361,18 @@
         <v>15</v>
       </c>
       <c r="G215" s="1" t="s">
-        <v>553</v>
+        <v>538</v>
       </c>
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B216" s="49" t="s">
-        <v>430</v>
+      <c r="B216" s="45" t="s">
+        <v>429</v>
       </c>
       <c r="C216" s="10" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D216" s="10">
         <v>3</v>
@@ -7378,21 +7384,21 @@
         <v>15</v>
       </c>
       <c r="G216" s="1" t="s">
-        <v>526</v>
+        <v>553</v>
       </c>
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B217" s="48" t="s">
-        <v>434</v>
-      </c>
-      <c r="C217" s="11" t="s">
-        <v>425</v>
-      </c>
-      <c r="D217" s="11">
-        <v>2</v>
+      <c r="B217" s="49" t="s">
+        <v>430</v>
+      </c>
+      <c r="C217" s="10" t="s">
+        <v>424</v>
+      </c>
+      <c r="D217" s="10">
+        <v>3</v>
       </c>
       <c r="E217" s="51" t="s">
         <v>435</v>
@@ -7401,7 +7407,7 @@
         <v>15</v>
       </c>
       <c r="G217" s="1" t="s">
-        <v>552</v>
+        <v>526</v>
       </c>
     </row>
     <row r="218" spans="1:7" x14ac:dyDescent="0.25">
@@ -7412,10 +7418,10 @@
         <v>434</v>
       </c>
       <c r="C218" s="11" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D218" s="11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E218" s="51" t="s">
         <v>435</v>
@@ -7424,21 +7430,21 @@
         <v>15</v>
       </c>
       <c r="G218" s="1" t="s">
-        <v>539</v>
+        <v>552</v>
       </c>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B219" s="47" t="s">
-        <v>431</v>
+      <c r="B219" s="48" t="s">
+        <v>434</v>
       </c>
       <c r="C219" s="11" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="D219" s="11">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E219" s="51" t="s">
         <v>435</v>
@@ -7447,41 +7453,41 @@
         <v>15</v>
       </c>
       <c r="G219" s="1" t="s">
-        <v>551</v>
+        <v>539</v>
       </c>
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" s="11" t="s">
-        <v>445</v>
+        <v>412</v>
       </c>
       <c r="B220" s="47" t="s">
         <v>431</v>
       </c>
-      <c r="C220" s="10" t="s">
-        <v>436</v>
-      </c>
-      <c r="D220" s="10">
-        <v>2</v>
-      </c>
-      <c r="E220" s="46" t="s">
-        <v>444</v>
+      <c r="C220" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="D220" s="11">
+        <v>10</v>
+      </c>
+      <c r="E220" s="51" t="s">
+        <v>435</v>
       </c>
       <c r="F220" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G220" s="1" t="s">
-        <v>529</v>
+        <v>551</v>
       </c>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" s="11" t="s">
-        <v>412</v>
-      </c>
-      <c r="B221" s="5" t="s">
-        <v>446</v>
+        <v>445</v>
+      </c>
+      <c r="B221" s="47" t="s">
+        <v>431</v>
       </c>
       <c r="C221" s="10" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D221" s="10">
         <v>2</v>
@@ -7493,7 +7499,7 @@
         <v>15</v>
       </c>
       <c r="G221" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.25">
@@ -7504,10 +7510,10 @@
         <v>446</v>
       </c>
       <c r="C222" s="10" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="D222" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E222" s="46" t="s">
         <v>444</v>
@@ -7526,10 +7532,10 @@
       <c r="B223" s="5" t="s">
         <v>446</v>
       </c>
-      <c r="C223" s="52" t="s">
-        <v>439</v>
-      </c>
-      <c r="D223" s="11">
+      <c r="C223" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="D223" s="10">
         <v>1</v>
       </c>
       <c r="E223" s="46" t="s">
@@ -7539,7 +7545,7 @@
         <v>15</v>
       </c>
       <c r="G223" s="1" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.25">
@@ -7549,8 +7555,8 @@
       <c r="B224" s="5" t="s">
         <v>446</v>
       </c>
-      <c r="C224" s="11" t="s">
-        <v>440</v>
+      <c r="C224" s="52" t="s">
+        <v>439</v>
       </c>
       <c r="D224" s="11">
         <v>1</v>
@@ -7562,21 +7568,21 @@
         <v>15</v>
       </c>
       <c r="G224" s="1" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B225" s="49" t="s">
-        <v>430</v>
-      </c>
-      <c r="C225" s="10" t="s">
-        <v>441</v>
-      </c>
-      <c r="D225" s="10">
-        <v>2</v>
+      <c r="B225" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="C225" s="11" t="s">
+        <v>440</v>
+      </c>
+      <c r="D225" s="11">
+        <v>1</v>
       </c>
       <c r="E225" s="46" t="s">
         <v>444</v>
@@ -7585,18 +7591,18 @@
         <v>15</v>
       </c>
       <c r="G225" s="1" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B226" s="45" t="s">
-        <v>431</v>
+      <c r="B226" s="49" t="s">
+        <v>430</v>
       </c>
       <c r="C226" s="10" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="D226" s="10">
         <v>2</v>
@@ -7608,64 +7614,64 @@
         <v>15</v>
       </c>
       <c r="G226" s="1" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A227" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="B227" s="45" t="s">
+        <v>431</v>
+      </c>
+      <c r="C227" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="D227" s="10">
+        <v>2</v>
+      </c>
+      <c r="E227" s="46" t="s">
+        <v>444</v>
+      </c>
+      <c r="F227" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G227" s="1" t="s">
         <v>541</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A227" s="22" t="s">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A228" s="22" t="s">
         <v>412</v>
       </c>
-      <c r="B227" s="53" t="s">
+      <c r="B228" s="53" t="s">
         <v>431</v>
       </c>
-      <c r="C227" s="17" t="s">
+      <c r="C228" s="17" t="s">
         <v>443</v>
       </c>
-      <c r="D227" s="17">
+      <c r="D228" s="17">
         <v>3</v>
       </c>
-      <c r="E227" s="54" t="s">
+      <c r="E228" s="54" t="s">
         <v>444</v>
       </c>
-      <c r="F227" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G227" s="27" t="s">
+      <c r="F228" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G228" s="27" t="s">
         <v>542</v>
-      </c>
-    </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A228" s="11" t="s">
-        <v>448</v>
-      </c>
-      <c r="B228" s="11" t="s">
-        <v>448</v>
-      </c>
-      <c r="C228" s="10" t="s">
-        <v>448</v>
-      </c>
-      <c r="D228" s="10">
-        <v>5</v>
-      </c>
-      <c r="E228" s="36" t="s">
-        <v>447</v>
-      </c>
-      <c r="F228" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G228" s="1" t="s">
-        <v>543</v>
       </c>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229" s="11" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B229" s="11" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C229" s="10" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D229" s="10">
         <v>5</v>
@@ -7677,21 +7683,21 @@
         <v>15</v>
       </c>
       <c r="G229" s="1" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230" s="11" t="s">
-        <v>432</v>
+        <v>449</v>
       </c>
       <c r="B230" s="11" t="s">
-        <v>432</v>
+        <v>449</v>
       </c>
       <c r="C230" s="10" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="D230" s="10">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E230" s="36" t="s">
         <v>447</v>
@@ -7700,7 +7706,7 @@
         <v>15</v>
       </c>
       <c r="G230" s="1" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.25">
@@ -7710,10 +7716,10 @@
       <c r="B231" s="11" t="s">
         <v>432</v>
       </c>
-      <c r="C231" s="11" t="s">
-        <v>451</v>
-      </c>
-      <c r="D231" s="11">
+      <c r="C231" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="D231" s="10">
         <v>1</v>
       </c>
       <c r="E231" s="36" t="s">
@@ -7727,49 +7733,49 @@
       </c>
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A232" s="22" t="s">
+      <c r="A232" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="B232" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="C232" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="D232" s="11">
+        <v>1</v>
+      </c>
+      <c r="E232" s="36" t="s">
+        <v>447</v>
+      </c>
+      <c r="F232" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G232" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A233" s="22" t="s">
         <v>453</v>
       </c>
-      <c r="B232" s="22" t="s">
+      <c r="B233" s="22" t="s">
         <v>511</v>
       </c>
-      <c r="C232" s="22" t="s">
+      <c r="C233" s="22" t="s">
         <v>452</v>
       </c>
-      <c r="D232" s="22">
+      <c r="D233" s="22">
         <v>1</v>
       </c>
-      <c r="E232" s="55" t="s">
+      <c r="E233" s="55" t="s">
         <v>447</v>
       </c>
-      <c r="F232" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G232" s="27" t="s">
+      <c r="F233" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G233" s="27" t="s">
         <v>545</v>
-      </c>
-    </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A233" s="11" t="s">
-        <v>454</v>
-      </c>
-      <c r="B233" s="11" t="s">
-        <v>454</v>
-      </c>
-      <c r="C233" s="10" t="s">
-        <v>455</v>
-      </c>
-      <c r="D233" s="10">
-        <v>100</v>
-      </c>
-      <c r="E233" s="56" t="s">
-        <v>480</v>
-      </c>
-      <c r="F233" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G233" s="1" t="s">
-        <v>549</v>
       </c>
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.25">
@@ -7780,10 +7786,10 @@
         <v>454</v>
       </c>
       <c r="C234" s="10" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="D234" s="10">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="E234" s="56" t="s">
         <v>480</v>
@@ -7791,7 +7797,9 @@
       <c r="F234" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G234" s="1"/>
+      <c r="G234" s="1" t="s">
+        <v>549</v>
+      </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235" s="11" t="s">
@@ -7801,10 +7809,10 @@
         <v>454</v>
       </c>
       <c r="C235" s="10" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D235" s="10">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="E235" s="56" t="s">
         <v>480</v>
@@ -7822,10 +7830,10 @@
         <v>454</v>
       </c>
       <c r="C236" s="10" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D236" s="10">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="E236" s="56" t="s">
         <v>480</v>
@@ -7843,10 +7851,10 @@
         <v>454</v>
       </c>
       <c r="C237" s="10" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D237" s="10">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E237" s="56" t="s">
         <v>480</v>
@@ -7864,10 +7872,10 @@
         <v>454</v>
       </c>
       <c r="C238" s="10" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="D238" s="10">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E238" s="56" t="s">
         <v>480</v>
@@ -7885,10 +7893,10 @@
         <v>454</v>
       </c>
       <c r="C239" s="10" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D239" s="10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E239" s="56" t="s">
         <v>480</v>
@@ -7896,9 +7904,7 @@
       <c r="F239" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G239" s="1" t="s">
-        <v>554</v>
-      </c>
+      <c r="G239" s="1"/>
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240" s="11" t="s">
@@ -7908,10 +7914,10 @@
         <v>454</v>
       </c>
       <c r="C240" s="10" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D240" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E240" s="56" t="s">
         <v>480</v>
@@ -7919,7 +7925,9 @@
       <c r="F240" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G240" s="1"/>
+      <c r="G240" s="1" t="s">
+        <v>554</v>
+      </c>
     </row>
     <row r="241" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A241" s="11" t="s">
@@ -7929,10 +7937,10 @@
         <v>454</v>
       </c>
       <c r="C241" s="10" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D241" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E241" s="56" t="s">
         <v>480</v>
@@ -7950,10 +7958,10 @@
         <v>454</v>
       </c>
       <c r="C242" s="10" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="D242" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E242" s="56" t="s">
         <v>480</v>
@@ -7971,10 +7979,10 @@
         <v>454</v>
       </c>
       <c r="C243" s="10" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D243" s="10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E243" s="56" t="s">
         <v>480</v>
@@ -7992,10 +8000,10 @@
         <v>454</v>
       </c>
       <c r="C244" s="10" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D244" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E244" s="56" t="s">
         <v>480</v>
@@ -8012,11 +8020,11 @@
       <c r="B245" s="11" t="s">
         <v>454</v>
       </c>
-      <c r="C245" s="11" t="s">
-        <v>467</v>
-      </c>
-      <c r="D245" s="11">
-        <v>1</v>
+      <c r="C245" s="10" t="s">
+        <v>466</v>
+      </c>
+      <c r="D245" s="10">
+        <v>2</v>
       </c>
       <c r="E245" s="56" t="s">
         <v>480</v>
@@ -8034,10 +8042,10 @@
         <v>454</v>
       </c>
       <c r="C246" s="11" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D246" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E246" s="56" t="s">
         <v>480</v>
@@ -8055,10 +8063,10 @@
         <v>454</v>
       </c>
       <c r="C247" s="11" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D247" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E247" s="56" t="s">
         <v>480</v>
@@ -8076,7 +8084,7 @@
         <v>454</v>
       </c>
       <c r="C248" s="11" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="D248" s="11">
         <v>1</v>
@@ -8097,10 +8105,10 @@
         <v>454</v>
       </c>
       <c r="C249" s="11" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D249" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E249" s="56" t="s">
         <v>480</v>
@@ -8118,10 +8126,10 @@
         <v>454</v>
       </c>
       <c r="C250" s="11" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="D250" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E250" s="56" t="s">
         <v>480</v>
@@ -8139,7 +8147,7 @@
         <v>454</v>
       </c>
       <c r="C251" s="11" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D251" s="11">
         <v>1</v>
@@ -8160,7 +8168,7 @@
         <v>454</v>
       </c>
       <c r="C252" s="11" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="D252" s="11">
         <v>1</v>
@@ -8181,7 +8189,7 @@
         <v>454</v>
       </c>
       <c r="C253" s="11" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D253" s="11">
         <v>1</v>
@@ -8202,10 +8210,10 @@
         <v>454</v>
       </c>
       <c r="C254" s="11" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D254" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E254" s="56" t="s">
         <v>480</v>
@@ -8223,10 +8231,10 @@
         <v>454</v>
       </c>
       <c r="C255" s="11" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D255" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E255" s="56" t="s">
         <v>480</v>
@@ -8234,9 +8242,7 @@
       <c r="F255" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G255" s="1" t="s">
-        <v>546</v>
-      </c>
+      <c r="G255" s="1"/>
     </row>
     <row r="256" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A256" s="11" t="s">
@@ -8246,10 +8252,10 @@
         <v>454</v>
       </c>
       <c r="C256" s="11" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D256" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E256" s="56" t="s">
         <v>480</v>
@@ -8258,7 +8264,7 @@
         <v>15</v>
       </c>
       <c r="G256" s="1" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.25">
@@ -8269,10 +8275,10 @@
         <v>454</v>
       </c>
       <c r="C257" s="11" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="D257" s="11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E257" s="56" t="s">
         <v>480</v>
@@ -8280,16 +8286,39 @@
       <c r="F257" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G257" s="1"/>
+      <c r="G257" s="1" t="s">
+        <v>548</v>
+      </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A258" s="1"/>
-      <c r="B258" s="1"/>
-      <c r="C258" s="1"/>
-      <c r="D258" s="1"/>
-      <c r="E258" s="1"/>
-      <c r="F258" s="1"/>
+      <c r="A258" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="B258" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="C258" s="11" t="s">
+        <v>479</v>
+      </c>
+      <c r="D258" s="11">
+        <v>1</v>
+      </c>
+      <c r="E258" s="56" t="s">
+        <v>480</v>
+      </c>
+      <c r="F258" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="G258" s="1"/>
+    </row>
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A259" s="1"/>
+      <c r="B259" s="1"/>
+      <c r="C259" s="1"/>
+      <c r="D259" s="1"/>
+      <c r="E259" s="1"/>
+      <c r="F259" s="1"/>
+      <c r="G259" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
banco de dados e tabela funcionando
</commit_message>
<xml_diff>
--- a/planilhas/estoque_lab_completa.xlsx
+++ b/planilhas/estoque_lab_completa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H258"/>
+  <dimension ref="A1:H260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10224,6 +10224,82 @@
         </is>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Conector Bcn Femea X Femea</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Conector Rf</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>CONECTOR BNC FXF</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>4</v>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Maleta preta de conectores de RF</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>A Maleta Fica Na Mesa Branca</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>SLOT ÚNICO GERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Conector Kre X Bnc Macho</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Conector Rf</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>KRE X BNC MACHO</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>4</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Maleta Preta de conectores de RF</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>A Maleta</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>SLOT ÚNICO GERAL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
backup do banco com numero errados
</commit_message>
<xml_diff>
--- a/planilhas/estoque_lab_completa.xlsx
+++ b/planilhas/estoque_lab_completa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H260"/>
+  <dimension ref="A1:H263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>85</v>
+        <v>170</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>480</v>
+        <v>960</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -934,7 +934,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>235</v>
+        <v>470</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>85</v>
+        <v>170</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>410</v>
+        <v>820</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1428,7 +1428,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>550</v>
+        <v>1100</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>95</v>
+        <v>190</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1580,7 +1580,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>490</v>
+        <v>980</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>285</v>
+        <v>570</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1656,7 +1656,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>180</v>
+        <v>360</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>535</v>
+        <v>1070</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1770,7 +1770,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>245</v>
+        <v>490</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>205</v>
+        <v>410</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>95</v>
+        <v>190</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>110</v>
+        <v>220</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>225</v>
+        <v>450</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -2036,7 +2036,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>595</v>
+        <v>1190</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -2112,7 +2112,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>260</v>
+        <v>520</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2264,7 +2264,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>425</v>
+        <v>850</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>275</v>
+        <v>550</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>595</v>
+        <v>1190</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2378,7 +2378,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2416,7 +2416,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2454,7 +2454,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>290</v>
+        <v>580</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2492,7 +2492,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2568,7 +2568,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2606,7 +2606,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2644,7 +2644,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>275</v>
+        <v>550</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>265</v>
+        <v>530</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>95</v>
+        <v>190</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -2796,7 +2796,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>350</v>
+        <v>700</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -2834,7 +2834,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2872,7 +2872,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>245</v>
+        <v>490</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2986,7 +2986,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -3024,7 +3024,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -3138,7 +3138,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -3176,7 +3176,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -3214,7 +3214,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -3404,7 +3404,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -3442,7 +3442,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -3480,7 +3480,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -3518,7 +3518,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -3556,7 +3556,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -3594,7 +3594,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -3632,7 +3632,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -3670,7 +3670,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -3708,7 +3708,7 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -3746,7 +3746,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -3784,7 +3784,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -3822,7 +3822,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -3860,7 +3860,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -3936,7 +3936,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -3974,7 +3974,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -4050,7 +4050,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -4126,7 +4126,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -4164,7 +4164,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -4202,7 +4202,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -4240,7 +4240,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -4278,7 +4278,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -4392,7 +4392,7 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>170</v>
+        <v>340</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -4430,7 +4430,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -4468,7 +4468,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -4506,7 +4506,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -4544,7 +4544,7 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -4582,7 +4582,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -4620,7 +4620,7 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>110</v>
+        <v>220</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -4658,7 +4658,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
@@ -4696,7 +4696,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -4734,7 +4734,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -4772,7 +4772,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -4810,7 +4810,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
@@ -4886,7 +4886,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
@@ -4924,7 +4924,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -5000,7 +5000,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -5038,7 +5038,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -5076,7 +5076,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>115</v>
+        <v>230</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -5152,7 +5152,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -5190,7 +5190,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -5228,7 +5228,7 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
@@ -5266,7 +5266,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
@@ -5304,7 +5304,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -5342,7 +5342,7 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -5380,7 +5380,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -5418,7 +5418,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>125</v>
+        <v>250</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -5456,7 +5456,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -5494,7 +5494,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -5532,7 +5532,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -5608,7 +5608,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
@@ -5646,7 +5646,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -5684,7 +5684,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>115</v>
+        <v>230</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -5722,7 +5722,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -5760,7 +5760,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>105</v>
+        <v>210</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -5836,7 +5836,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
@@ -5874,7 +5874,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F144" t="inlineStr">
         <is>
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
@@ -5950,7 +5950,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F146" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -6026,7 +6026,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
@@ -6064,7 +6064,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
@@ -6102,7 +6102,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
@@ -6140,7 +6140,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
@@ -6178,7 +6178,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
@@ -6216,7 +6216,7 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
@@ -6254,7 +6254,7 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
@@ -6292,7 +6292,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -6330,7 +6330,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
@@ -6444,7 +6444,7 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
@@ -6482,7 +6482,7 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F161" t="inlineStr">
         <is>
@@ -6558,7 +6558,7 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F162" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F163" t="inlineStr">
         <is>
@@ -6634,7 +6634,7 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
@@ -6672,7 +6672,7 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F165" t="inlineStr">
         <is>
@@ -6710,7 +6710,7 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F167" t="inlineStr">
         <is>
@@ -6786,7 +6786,7 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F168" t="inlineStr">
         <is>
@@ -6824,7 +6824,7 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F169" t="inlineStr">
         <is>
@@ -6862,7 +6862,7 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F170" t="inlineStr">
         <is>
@@ -6900,7 +6900,7 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>135</v>
+        <v>270</v>
       </c>
       <c r="F171" t="inlineStr">
         <is>
@@ -6938,7 +6938,7 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F172" t="inlineStr">
         <is>
@@ -6976,7 +6976,7 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F173" t="inlineStr">
         <is>
@@ -7014,7 +7014,7 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
@@ -7052,7 +7052,7 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F175" t="inlineStr">
         <is>
@@ -7090,7 +7090,7 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F176" t="inlineStr">
         <is>
@@ -7128,7 +7128,7 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F177" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F178" t="inlineStr">
         <is>
@@ -7204,7 +7204,7 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F179" t="inlineStr">
         <is>
@@ -7242,7 +7242,7 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F180" t="inlineStr">
         <is>
@@ -7280,7 +7280,7 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="F181" t="inlineStr">
         <is>
@@ -7318,7 +7318,7 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F182" t="inlineStr">
         <is>
@@ -7356,7 +7356,7 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F183" t="inlineStr">
         <is>
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="F184" t="inlineStr">
         <is>
@@ -7432,7 +7432,7 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="F185" t="inlineStr">
         <is>
@@ -7470,7 +7470,7 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="F186" t="inlineStr">
         <is>
@@ -7508,7 +7508,7 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F187" t="inlineStr">
         <is>
@@ -7546,7 +7546,7 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F188" t="inlineStr">
         <is>
@@ -7584,7 +7584,7 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F189" t="inlineStr">
         <is>
@@ -7622,7 +7622,7 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F190" t="inlineStr">
         <is>
@@ -7660,7 +7660,7 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F191" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F192" t="inlineStr">
         <is>
@@ -7736,7 +7736,7 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F193" t="inlineStr">
         <is>
@@ -7774,7 +7774,7 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F194" t="inlineStr">
         <is>
@@ -7812,7 +7812,7 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F195" t="inlineStr">
         <is>
@@ -7850,7 +7850,7 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F196" t="inlineStr">
         <is>
@@ -7888,7 +7888,7 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F197" t="inlineStr">
         <is>
@@ -7926,7 +7926,7 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F198" t="inlineStr">
         <is>
@@ -7964,7 +7964,7 @@
         </is>
       </c>
       <c r="E199" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="F199" t="inlineStr">
         <is>
@@ -8002,7 +8002,7 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F200" t="inlineStr">
         <is>
@@ -8040,7 +8040,7 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F201" t="inlineStr">
         <is>
@@ -8078,7 +8078,7 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F202" t="inlineStr">
         <is>
@@ -8116,7 +8116,7 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F203" t="inlineStr">
         <is>
@@ -8154,7 +8154,7 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F204" t="inlineStr">
         <is>
@@ -8192,7 +8192,7 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F205" t="inlineStr">
         <is>
@@ -8230,7 +8230,7 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F206" t="inlineStr">
         <is>
@@ -8268,7 +8268,7 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F207" t="inlineStr">
         <is>
@@ -8306,7 +8306,7 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F208" t="inlineStr">
         <is>
@@ -8344,7 +8344,7 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="F209" t="inlineStr">
         <is>
@@ -8382,7 +8382,7 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F210" t="inlineStr">
         <is>
@@ -8420,7 +8420,7 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F211" t="inlineStr">
         <is>
@@ -8458,7 +8458,7 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F212" t="inlineStr">
         <is>
@@ -8496,7 +8496,7 @@
         </is>
       </c>
       <c r="E213" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F213" t="inlineStr">
         <is>
@@ -8534,7 +8534,7 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F214" t="inlineStr">
         <is>
@@ -8572,7 +8572,7 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F215" t="inlineStr">
         <is>
@@ -8610,7 +8610,7 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F216" t="inlineStr">
         <is>
@@ -8648,7 +8648,7 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F217" t="inlineStr">
         <is>
@@ -8686,7 +8686,7 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F218" t="inlineStr">
         <is>
@@ -8724,7 +8724,7 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F219" t="inlineStr">
         <is>
@@ -8762,7 +8762,7 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F220" t="inlineStr">
         <is>
@@ -8800,7 +8800,7 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F221" t="inlineStr">
         <is>
@@ -8838,7 +8838,7 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F222" t="inlineStr">
         <is>
@@ -8876,7 +8876,7 @@
         </is>
       </c>
       <c r="E223" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F223" t="inlineStr">
         <is>
@@ -8914,7 +8914,7 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F224" t="inlineStr">
         <is>
@@ -8952,7 +8952,7 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F225" t="inlineStr">
         <is>
@@ -8990,7 +8990,7 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F226" t="inlineStr">
         <is>
@@ -9028,7 +9028,7 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F227" t="inlineStr">
         <is>
@@ -9066,7 +9066,7 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F228" t="inlineStr">
         <is>
@@ -9104,7 +9104,7 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F229" t="inlineStr">
         <is>
@@ -9142,7 +9142,7 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F230" t="inlineStr">
         <is>
@@ -9180,7 +9180,7 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F231" t="inlineStr">
         <is>
@@ -9218,7 +9218,7 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
@@ -9256,7 +9256,7 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>460</v>
+        <v>920</v>
       </c>
       <c r="F233" t="inlineStr">
         <is>
@@ -9294,7 +9294,7 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>345</v>
+        <v>690</v>
       </c>
       <c r="F234" t="inlineStr">
         <is>
@@ -9332,7 +9332,7 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="F235" t="inlineStr">
         <is>
@@ -9370,7 +9370,7 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="F236" t="inlineStr">
         <is>
@@ -9408,7 +9408,7 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F237" t="inlineStr">
         <is>
@@ -9446,7 +9446,7 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F238" t="inlineStr">
         <is>
@@ -9484,7 +9484,7 @@
         </is>
       </c>
       <c r="E239" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F239" t="inlineStr">
         <is>
@@ -9522,7 +9522,7 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F240" t="inlineStr">
         <is>
@@ -9560,7 +9560,7 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F241" t="inlineStr">
         <is>
@@ -9598,7 +9598,7 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F242" t="inlineStr">
         <is>
@@ -9636,7 +9636,7 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F243" t="inlineStr">
         <is>
@@ -9674,7 +9674,7 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F244" t="inlineStr">
         <is>
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F245" t="inlineStr">
         <is>
@@ -9750,7 +9750,7 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F246" t="inlineStr">
         <is>
@@ -9788,7 +9788,7 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F247" t="inlineStr">
         <is>
@@ -9826,7 +9826,7 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F248" t="inlineStr">
         <is>
@@ -9864,7 +9864,7 @@
         </is>
       </c>
       <c r="E249" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F249" t="inlineStr">
         <is>
@@ -9902,7 +9902,7 @@
         </is>
       </c>
       <c r="E250" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F250" t="inlineStr">
         <is>
@@ -9940,7 +9940,7 @@
         </is>
       </c>
       <c r="E251" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F251" t="inlineStr">
         <is>
@@ -9978,7 +9978,7 @@
         </is>
       </c>
       <c r="E252" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F252" t="inlineStr">
         <is>
@@ -10016,7 +10016,7 @@
         </is>
       </c>
       <c r="E253" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F253" t="inlineStr">
         <is>
@@ -10054,7 +10054,7 @@
         </is>
       </c>
       <c r="E254" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F254" t="inlineStr">
         <is>
@@ -10092,7 +10092,7 @@
         </is>
       </c>
       <c r="E255" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F255" t="inlineStr">
         <is>
@@ -10130,7 +10130,7 @@
         </is>
       </c>
       <c r="E256" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F256" t="inlineStr">
         <is>
@@ -10168,7 +10168,7 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="E259" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F259" t="inlineStr">
         <is>
@@ -10282,21 +10282,135 @@
         </is>
       </c>
       <c r="E260" t="n">
+        <v>8</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Maleta Preta de conectores de RF</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>A Maleta</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>SLOT ÚNICO GERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Conector N De Carga</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Conectores</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>CONECTOR N COM CARGA DE 50 Ω</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>2</v>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Maleta preta de conectores</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Mesa Branca</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>SLOT UNICO GERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Conector Bnc T Fxfxm</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Conector Rf</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>BNT EM T FXFXM</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
         <v>4</v>
       </c>
-      <c r="F260" t="inlineStr">
-        <is>
-          <t>Maleta Preta de conectores de RF</t>
-        </is>
-      </c>
-      <c r="G260" t="inlineStr">
-        <is>
-          <t>A Maleta</t>
-        </is>
-      </c>
-      <c r="H260" t="inlineStr">
-        <is>
-          <t>SLOT ÚNICO GERAL</t>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Caixa dos conectores</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Armário</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>SLOT A</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Conector Bnc F 90º X Sma M</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Conector Rf</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>BNC F 90º X SMA M</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>4</v>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Caixa dos conectores</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Armário</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>SLOT A</t>
         </is>
       </c>
     </row>

</xml_diff>